<commit_message>
fix(kqkd): reconcile Month 7 LNTT 830, THH Cum 2376, ITSS/VPSM equity and finalize template
</commit_message>
<xml_diff>
--- a/Template_Bao_Cao_KQKD_Hop_Nhat_VPS.xlsx
+++ b/Template_Bao_Cao_KQKD_Hop_Nhat_VPS.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -189,16 +189,16 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -207,15 +207,15 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -225,12 +225,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -240,16 +240,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -258,13 +258,13 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -795,30 +795,32 @@
           <t>MIỀN BẮC</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="10" t="inlineStr"/>
-      <c r="E7" s="11" t="n">
+      <c r="C7" s="10" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D7" s="11" t="inlineStr"/>
+      <c r="E7" s="12" t="n">
         <v>0.1</v>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="12" t="n">
+      <c r="F7" s="11" t="inlineStr"/>
+      <c r="G7" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr"/>
+      <c r="H7" s="11" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr"/>
       <c r="J7" s="13" t="n">
         <v>-89</v>
       </c>
-      <c r="K7" s="10" t="inlineStr"/>
-      <c r="L7" s="11" t="n">
+      <c r="K7" s="11" t="inlineStr"/>
+      <c r="L7" s="12" t="n">
         <v>0.21</v>
       </c>
-      <c r="M7" s="10" t="inlineStr"/>
-      <c r="N7" s="12" t="n">
+      <c r="M7" s="11" t="inlineStr"/>
+      <c r="N7" s="10" t="n">
         <v>335</v>
       </c>
-      <c r="O7" s="10" t="inlineStr"/>
-      <c r="P7" s="12" t="n">
+      <c r="O7" s="11" t="inlineStr"/>
+      <c r="P7" s="10" t="n">
         <v>7731</v>
       </c>
       <c r="Q7" s="13" t="n">
@@ -867,7 +869,7 @@
         <v>57</v>
       </c>
       <c r="Q8" s="16" t="n">
-        <v>286</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="9">
@@ -903,7 +905,9 @@
       <c r="L9" s="22" t="n">
         <v>0.36</v>
       </c>
-      <c r="M9" s="21" t="inlineStr"/>
+      <c r="M9" s="23" t="n">
+        <v>5747</v>
+      </c>
       <c r="N9" s="23" t="n">
         <v>54</v>
       </c>
@@ -977,20 +981,20 @@
         <v>0.5</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>146.7</v>
+        <v>144.7</v>
       </c>
       <c r="G11" s="26" t="inlineStr"/>
       <c r="H11" s="26" t="inlineStr"/>
       <c r="I11" s="26" t="inlineStr"/>
       <c r="J11" s="26" t="inlineStr"/>
       <c r="K11" s="27" t="n">
-        <v>2054.4</v>
+        <v>2054.6</v>
       </c>
       <c r="L11" s="28" t="n">
         <v>0.51</v>
       </c>
       <c r="M11" s="27" t="n">
-        <v>1048.5</v>
+        <v>1058</v>
       </c>
       <c r="N11" s="26" t="inlineStr"/>
       <c r="O11" s="26" t="inlineStr"/>
@@ -1055,7 +1059,7 @@
         <v>0.61</v>
       </c>
       <c r="F13" s="27" t="n">
-        <v>141.6</v>
+        <v>141</v>
       </c>
       <c r="G13" s="26" t="inlineStr"/>
       <c r="H13" s="26" t="inlineStr"/>
@@ -1068,7 +1072,7 @@
         <v>0.51</v>
       </c>
       <c r="M13" s="27" t="n">
-        <v>738.9</v>
+        <v>737.6</v>
       </c>
       <c r="N13" s="26" t="inlineStr"/>
       <c r="O13" s="26" t="inlineStr"/>
@@ -1131,13 +1135,13 @@
       </c>
       <c r="C15" s="21" t="inlineStr"/>
       <c r="D15" s="23" t="n">
-        <v>1100</v>
+        <v>1139</v>
       </c>
       <c r="E15" s="22" t="n">
         <v>0.15</v>
       </c>
       <c r="F15" s="23" t="n">
-        <v>165</v>
+        <v>174.6</v>
       </c>
       <c r="G15" s="21" t="inlineStr"/>
       <c r="H15" s="23" t="n">
@@ -1149,14 +1153,12 @@
       <c r="J15" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="K15" s="23" t="n">
-        <v>12937.5</v>
-      </c>
+      <c r="K15" s="21" t="inlineStr"/>
       <c r="L15" s="22" t="n">
         <v>0.08</v>
       </c>
       <c r="M15" s="23" t="n">
-        <v>1035</v>
+        <v>1034.7</v>
       </c>
       <c r="N15" s="23" t="n">
         <v>9</v>
@@ -1208,11 +1210,15 @@
       <c r="L16" s="22" t="n">
         <v>0.09</v>
       </c>
-      <c r="M16" s="21" t="inlineStr"/>
+      <c r="M16" s="23" t="n">
+        <v>2275.1</v>
+      </c>
       <c r="N16" s="23" t="n">
         <v>271</v>
       </c>
-      <c r="O16" s="21" t="inlineStr"/>
+      <c r="O16" s="23" t="n">
+        <v>2438</v>
+      </c>
       <c r="P16" s="23" t="n">
         <v>10</v>
       </c>
@@ -1255,9 +1261,13 @@
       </c>
       <c r="M17" s="21" t="inlineStr"/>
       <c r="N17" s="21" t="inlineStr"/>
-      <c r="O17" s="21" t="inlineStr"/>
+      <c r="O17" s="23" t="n">
+        <v>3342</v>
+      </c>
       <c r="P17" s="21" t="inlineStr"/>
-      <c r="Q17" s="21" t="inlineStr"/>
+      <c r="Q17" s="23" t="n">
+        <v>2038</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
@@ -1292,9 +1302,13 @@
       <c r="L18" s="18" t="n">
         <v>0.21</v>
       </c>
-      <c r="M18" s="17" t="inlineStr"/>
+      <c r="M18" s="16" t="n">
+        <v>8562</v>
+      </c>
       <c r="N18" s="17" t="inlineStr"/>
-      <c r="O18" s="17" t="inlineStr"/>
+      <c r="O18" s="16" t="n">
+        <v>6903</v>
+      </c>
       <c r="P18" s="16" t="n">
         <v>13</v>
       </c>
@@ -1509,7 +1523,9 @@
           <t>ITSS</t>
         </is>
       </c>
-      <c r="C23" s="17" t="inlineStr"/>
+      <c r="C23" s="16" t="n">
+        <v>5000</v>
+      </c>
       <c r="D23" s="16" t="n">
         <v>524</v>
       </c>
@@ -1536,7 +1552,7 @@
         <v>0.35</v>
       </c>
       <c r="M23" s="16" t="n">
-        <v>1020</v>
+        <v>1028</v>
       </c>
       <c r="N23" s="17" t="inlineStr"/>
       <c r="O23" s="16" t="n">
@@ -1571,14 +1587,20 @@
       <c r="G24" s="17" t="inlineStr"/>
       <c r="H24" s="17" t="inlineStr"/>
       <c r="I24" s="17" t="inlineStr"/>
-      <c r="J24" s="17" t="inlineStr"/>
+      <c r="J24" s="30" t="n">
+        <v>-828</v>
+      </c>
       <c r="K24" s="17" t="inlineStr"/>
       <c r="L24" s="17" t="inlineStr"/>
       <c r="M24" s="17" t="inlineStr"/>
       <c r="N24" s="17" t="inlineStr"/>
       <c r="O24" s="17" t="inlineStr"/>
-      <c r="P24" s="17" t="inlineStr"/>
-      <c r="Q24" s="17" t="inlineStr"/>
+      <c r="P24" s="16" t="n">
+        <v>7665</v>
+      </c>
+      <c r="Q24" s="30" t="n">
+        <v>-4447</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
@@ -1593,7 +1615,7 @@
       </c>
       <c r="C25" s="26" t="inlineStr"/>
       <c r="D25" s="27" t="n">
-        <v>14351</v>
+        <v>14951</v>
       </c>
       <c r="E25" s="28" t="n">
         <v>0.031</v>
@@ -1673,7 +1695,7 @@
       </c>
       <c r="N26" s="26" t="inlineStr"/>
       <c r="O26" s="27" t="n">
-        <v>3727</v>
+        <v>9727</v>
       </c>
       <c r="P26" s="27" t="n">
         <v>4933</v>
@@ -2143,45 +2165,45 @@
           <t>VPS MIỀN TRUNG</t>
         </is>
       </c>
-      <c r="C37" s="12" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D37" s="12" t="n">
+      <c r="C37" s="10" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D37" s="10" t="n">
         <v>1674</v>
       </c>
-      <c r="E37" s="11" t="n">
+      <c r="E37" s="12" t="n">
         <v>0.14</v>
       </c>
-      <c r="F37" s="12" t="n">
+      <c r="F37" s="10" t="n">
         <v>239</v>
       </c>
-      <c r="G37" s="10" t="inlineStr"/>
-      <c r="H37" s="12" t="n">
+      <c r="G37" s="11" t="inlineStr"/>
+      <c r="H37" s="10" t="n">
         <v>220</v>
       </c>
-      <c r="I37" s="12" t="n">
+      <c r="I37" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="J37" s="12" t="n">
+      <c r="J37" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="K37" s="12" t="n">
-        <v>11252</v>
-      </c>
-      <c r="L37" s="11" t="n">
+      <c r="K37" s="10" t="n">
+        <v>11251</v>
+      </c>
+      <c r="L37" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="M37" s="12" t="n">
-        <v>2266</v>
-      </c>
-      <c r="N37" s="10" t="inlineStr"/>
-      <c r="O37" s="12" t="n">
+      <c r="M37" s="10" t="n">
+        <v>2267</v>
+      </c>
+      <c r="N37" s="11" t="inlineStr"/>
+      <c r="O37" s="10" t="n">
         <v>1515</v>
       </c>
-      <c r="P37" s="12" t="n">
+      <c r="P37" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="Q37" s="12" t="n">
+      <c r="Q37" s="10" t="n">
         <v>828</v>
       </c>
     </row>
@@ -2305,7 +2327,7 @@
         <v>0.43</v>
       </c>
       <c r="F41" s="27" t="n">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="G41" s="26" t="inlineStr"/>
       <c r="H41" s="26" t="inlineStr"/>
@@ -2457,7 +2479,7 @@
         <v>1161</v>
       </c>
       <c r="J45" s="33" t="n">
-        <v>530</v>
+        <v>830</v>
       </c>
       <c r="K45" s="34" t="inlineStr"/>
       <c r="L45" s="35" t="n">

</xml_diff>

<commit_message>
fix(kqkd): update Vốn ĐT 93000, Month 7 DS 43128, Cum DS 208724 and exact group sums
</commit_message>
<xml_diff>
--- a/Template_Bao_Cao_KQKD_Hop_Nhat_VPS.xlsx
+++ b/Template_Bao_Cao_KQKD_Hop_Nhat_VPS.xlsx
@@ -160,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -192,66 +192,66 @@
     <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -259,9 +259,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -796,1361 +793,1423 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>80000</v>
-      </c>
-      <c r="D7" s="11" t="inlineStr"/>
-      <c r="E7" s="12" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>41454</v>
+      </c>
+      <c r="E7" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="F7" s="11" t="inlineStr"/>
+      <c r="F7" s="10" t="n">
+        <v>6070</v>
+      </c>
       <c r="G7" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="11" t="inlineStr"/>
-      <c r="I7" s="11" t="inlineStr"/>
-      <c r="J7" s="13" t="n">
+      <c r="H7" s="10" t="n">
+        <v>6865</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>1095</v>
+      </c>
+      <c r="J7" s="12" t="n">
         <v>-89</v>
       </c>
-      <c r="K7" s="11" t="inlineStr"/>
-      <c r="L7" s="12" t="n">
+      <c r="K7" s="10" t="n">
+        <v>197473</v>
+      </c>
+      <c r="L7" s="11" t="n">
         <v>0.21</v>
       </c>
-      <c r="M7" s="11" t="inlineStr"/>
+      <c r="M7" s="10" t="n">
+        <v>44982</v>
+      </c>
       <c r="N7" s="10" t="n">
         <v>335</v>
       </c>
-      <c r="O7" s="11" t="inlineStr"/>
+      <c r="O7" s="10" t="n">
+        <v>49241</v>
+      </c>
       <c r="P7" s="10" t="n">
         <v>7731</v>
       </c>
-      <c r="Q7" s="13" t="n">
+      <c r="Q7" s="12" t="n">
         <v>-234</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>THH (Tân Hồng Hà)</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="15" t="n">
         <v>50000</v>
       </c>
-      <c r="D8" s="17" t="inlineStr"/>
-      <c r="E8" s="18" t="n">
+      <c r="D8" s="15" t="n">
+        <v>8804</v>
+      </c>
+      <c r="E8" s="16" t="n">
         <v>0.18</v>
       </c>
-      <c r="F8" s="17" t="inlineStr"/>
-      <c r="G8" s="16" t="n">
+      <c r="F8" s="15" t="n">
+        <v>1568</v>
+      </c>
+      <c r="G8" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="17" t="inlineStr"/>
-      <c r="I8" s="16" t="n">
+      <c r="H8" s="15" t="n">
+        <v>1341</v>
+      </c>
+      <c r="I8" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="J8" s="16" t="n">
+      <c r="J8" s="15" t="n">
         <v>245</v>
       </c>
-      <c r="K8" s="17" t="inlineStr"/>
-      <c r="L8" s="18" t="n">
+      <c r="K8" s="15" t="n">
+        <v>66583</v>
+      </c>
+      <c r="L8" s="16" t="n">
         <v>0.21</v>
       </c>
-      <c r="M8" s="17" t="inlineStr"/>
-      <c r="N8" s="16" t="n">
+      <c r="M8" s="15" t="n">
+        <v>10082</v>
+      </c>
+      <c r="N8" s="15" t="n">
         <v>335</v>
       </c>
-      <c r="O8" s="17" t="inlineStr"/>
-      <c r="P8" s="16" t="n">
+      <c r="O8" s="15" t="n">
+        <v>12453</v>
+      </c>
+      <c r="P8" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="Q8" s="16" t="n">
+      <c r="Q8" s="15" t="n">
         <v>2376</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  Khối dịch vụ kỹ thuật</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr"/>
-      <c r="D9" s="21" t="inlineStr"/>
-      <c r="E9" s="22" t="n">
+      <c r="C9" s="19" t="inlineStr"/>
+      <c r="D9" s="20" t="n">
+        <v>2578</v>
+      </c>
+      <c r="E9" s="21" t="n">
         <v>0.335</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="20" t="n">
         <v>864</v>
       </c>
-      <c r="G9" s="21" t="inlineStr"/>
-      <c r="H9" s="23" t="n">
+      <c r="G9" s="19" t="inlineStr"/>
+      <c r="H9" s="20" t="n">
         <v>798</v>
       </c>
-      <c r="I9" s="23" t="n">
+      <c r="I9" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="23" t="n">
+      <c r="J9" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="K9" s="21" t="inlineStr"/>
-      <c r="L9" s="22" t="n">
+      <c r="K9" s="20" t="n">
+        <v>16146</v>
+      </c>
+      <c r="L9" s="21" t="n">
         <v>0.36</v>
       </c>
-      <c r="M9" s="23" t="n">
+      <c r="M9" s="20" t="n">
         <v>5747</v>
       </c>
-      <c r="N9" s="23" t="n">
+      <c r="N9" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="O9" s="23" t="n">
+      <c r="O9" s="20" t="n">
         <v>5516</v>
       </c>
-      <c r="P9" s="23" t="n">
+      <c r="P9" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="Q9" s="23" t="n">
+      <c r="Q9" s="20" t="n">
         <v>286</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>a.1</t>
         </is>
       </c>
-      <c r="B10" s="25" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Tổ Dịch vụ</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr"/>
-      <c r="D10" s="27" t="n">
+      <c r="C10" s="24" t="inlineStr"/>
+      <c r="D10" s="25" t="n">
         <v>1346</v>
       </c>
-      <c r="E10" s="28" t="n">
+      <c r="E10" s="26" t="n">
         <v>0.26</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="25" t="n">
         <v>347.5</v>
       </c>
-      <c r="G10" s="26" t="inlineStr"/>
-      <c r="H10" s="26" t="inlineStr"/>
-      <c r="I10" s="26" t="inlineStr"/>
-      <c r="J10" s="26" t="inlineStr"/>
-      <c r="K10" s="27" t="n">
+      <c r="G10" s="24" t="inlineStr"/>
+      <c r="H10" s="24" t="inlineStr"/>
+      <c r="I10" s="24" t="inlineStr"/>
+      <c r="J10" s="24" t="inlineStr"/>
+      <c r="K10" s="25" t="n">
         <v>8304.5</v>
       </c>
-      <c r="L10" s="28" t="n">
+      <c r="L10" s="26" t="n">
         <v>0.33</v>
       </c>
-      <c r="M10" s="27" t="n">
+      <c r="M10" s="25" t="n">
         <v>2745.2</v>
       </c>
-      <c r="N10" s="27" t="n">
+      <c r="N10" s="25" t="n">
         <v>53</v>
       </c>
-      <c r="O10" s="26" t="inlineStr"/>
-      <c r="P10" s="26" t="inlineStr"/>
-      <c r="Q10" s="26" t="inlineStr"/>
+      <c r="O10" s="24" t="inlineStr"/>
+      <c r="P10" s="24" t="inlineStr"/>
+      <c r="Q10" s="24" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>a.2</t>
         </is>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Tổ mực in</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr"/>
-      <c r="D11" s="27" t="n">
+      <c r="C11" s="24" t="inlineStr"/>
+      <c r="D11" s="25" t="n">
         <v>292</v>
       </c>
-      <c r="E11" s="28" t="n">
+      <c r="E11" s="26" t="n">
         <v>0.5</v>
       </c>
-      <c r="F11" s="27" t="n">
+      <c r="F11" s="25" t="n">
         <v>144.7</v>
       </c>
-      <c r="G11" s="26" t="inlineStr"/>
-      <c r="H11" s="26" t="inlineStr"/>
-      <c r="I11" s="26" t="inlineStr"/>
-      <c r="J11" s="26" t="inlineStr"/>
-      <c r="K11" s="27" t="n">
+      <c r="G11" s="24" t="inlineStr"/>
+      <c r="H11" s="24" t="inlineStr"/>
+      <c r="I11" s="24" t="inlineStr"/>
+      <c r="J11" s="24" t="inlineStr"/>
+      <c r="K11" s="25" t="n">
         <v>2054.6</v>
       </c>
-      <c r="L11" s="28" t="n">
+      <c r="L11" s="26" t="n">
         <v>0.51</v>
       </c>
-      <c r="M11" s="27" t="n">
+      <c r="M11" s="25" t="n">
         <v>1058</v>
       </c>
-      <c r="N11" s="26" t="inlineStr"/>
-      <c r="O11" s="26" t="inlineStr"/>
-      <c r="P11" s="26" t="inlineStr"/>
-      <c r="Q11" s="26" t="inlineStr"/>
+      <c r="N11" s="24" t="inlineStr"/>
+      <c r="O11" s="24" t="inlineStr"/>
+      <c r="P11" s="24" t="inlineStr"/>
+      <c r="Q11" s="24" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>a.3</t>
         </is>
       </c>
-      <c r="B12" s="25" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Thuê máy</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr"/>
-      <c r="D12" s="27" t="n">
+      <c r="C12" s="24" t="inlineStr"/>
+      <c r="D12" s="25" t="n">
         <v>605</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="26" t="n">
         <v>0.38</v>
       </c>
-      <c r="F12" s="27" t="n">
+      <c r="F12" s="25" t="n">
         <v>231.1</v>
       </c>
-      <c r="G12" s="26" t="inlineStr"/>
-      <c r="H12" s="26" t="inlineStr"/>
-      <c r="I12" s="26" t="inlineStr"/>
-      <c r="J12" s="26" t="inlineStr"/>
-      <c r="K12" s="27" t="n">
+      <c r="G12" s="24" t="inlineStr"/>
+      <c r="H12" s="24" t="inlineStr"/>
+      <c r="I12" s="24" t="inlineStr"/>
+      <c r="J12" s="24" t="inlineStr"/>
+      <c r="K12" s="25" t="n">
         <v>3654.1</v>
       </c>
-      <c r="L12" s="28" t="n">
+      <c r="L12" s="26" t="n">
         <v>0.33</v>
       </c>
-      <c r="M12" s="27" t="n">
+      <c r="M12" s="25" t="n">
         <v>1192.3</v>
       </c>
-      <c r="N12" s="26" t="inlineStr"/>
-      <c r="O12" s="26" t="inlineStr"/>
-      <c r="P12" s="26" t="inlineStr"/>
-      <c r="Q12" s="26" t="inlineStr"/>
+      <c r="N12" s="24" t="inlineStr"/>
+      <c r="O12" s="24" t="inlineStr"/>
+      <c r="P12" s="24" t="inlineStr"/>
+      <c r="Q12" s="24" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>a.4</t>
         </is>
       </c>
-      <c r="B13" s="25" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Metercharge</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr"/>
-      <c r="D13" s="27" t="n">
+      <c r="C13" s="24" t="inlineStr"/>
+      <c r="D13" s="25" t="n">
         <v>233</v>
       </c>
-      <c r="E13" s="28" t="n">
+      <c r="E13" s="26" t="n">
         <v>0.61</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="25" t="n">
         <v>141</v>
       </c>
-      <c r="G13" s="26" t="inlineStr"/>
-      <c r="H13" s="26" t="inlineStr"/>
-      <c r="I13" s="26" t="inlineStr"/>
-      <c r="J13" s="26" t="inlineStr"/>
-      <c r="K13" s="27" t="n">
+      <c r="G13" s="24" t="inlineStr"/>
+      <c r="H13" s="24" t="inlineStr"/>
+      <c r="I13" s="24" t="inlineStr"/>
+      <c r="J13" s="24" t="inlineStr"/>
+      <c r="K13" s="25" t="n">
         <v>1459.2</v>
       </c>
-      <c r="L13" s="28" t="n">
+      <c r="L13" s="26" t="n">
         <v>0.51</v>
       </c>
-      <c r="M13" s="27" t="n">
+      <c r="M13" s="25" t="n">
         <v>737.6</v>
       </c>
-      <c r="N13" s="26" t="inlineStr"/>
-      <c r="O13" s="26" t="inlineStr"/>
-      <c r="P13" s="26" t="inlineStr"/>
-      <c r="Q13" s="26" t="inlineStr"/>
+      <c r="N13" s="24" t="inlineStr"/>
+      <c r="O13" s="24" t="inlineStr"/>
+      <c r="P13" s="24" t="inlineStr"/>
+      <c r="Q13" s="24" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>a.5</t>
         </is>
       </c>
-      <c r="B14" s="25" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Kinh doanh Online</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr"/>
-      <c r="D14" s="27" t="n">
+      <c r="C14" s="24" t="inlineStr"/>
+      <c r="D14" s="25" t="n">
         <v>102</v>
       </c>
-      <c r="E14" s="28" t="n">
+      <c r="E14" s="26" t="n">
         <v>-0.01</v>
       </c>
-      <c r="F14" s="29" t="n">
+      <c r="F14" s="27" t="n">
         <v>-0.6</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="26" t="inlineStr"/>
-      <c r="I14" s="26" t="inlineStr"/>
-      <c r="J14" s="26" t="inlineStr"/>
-      <c r="K14" s="27" t="n">
+      <c r="H14" s="24" t="inlineStr"/>
+      <c r="I14" s="24" t="inlineStr"/>
+      <c r="J14" s="24" t="inlineStr"/>
+      <c r="K14" s="25" t="n">
         <v>673.4</v>
       </c>
-      <c r="L14" s="28" t="n">
+      <c r="L14" s="26" t="n">
         <v>0.02</v>
       </c>
-      <c r="M14" s="27" t="n">
+      <c r="M14" s="25" t="n">
         <v>14.1</v>
       </c>
-      <c r="N14" s="27" t="n">
+      <c r="N14" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="O14" s="26" t="inlineStr"/>
-      <c r="P14" s="26" t="inlineStr"/>
-      <c r="Q14" s="26" t="inlineStr"/>
+      <c r="O14" s="24" t="inlineStr"/>
+      <c r="P14" s="24" t="inlineStr"/>
+      <c r="Q14" s="24" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  Kinh doanh tổng hợp</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr"/>
-      <c r="D15" s="23" t="n">
+      <c r="C15" s="19" t="inlineStr"/>
+      <c r="D15" s="20" t="n">
         <v>1139</v>
       </c>
-      <c r="E15" s="22" t="n">
+      <c r="E15" s="21" t="n">
         <v>0.15</v>
       </c>
-      <c r="F15" s="23" t="n">
+      <c r="F15" s="20" t="n">
         <v>174.6</v>
       </c>
-      <c r="G15" s="21" t="inlineStr"/>
-      <c r="H15" s="23" t="n">
+      <c r="G15" s="19" t="inlineStr"/>
+      <c r="H15" s="20" t="n">
         <v>165</v>
       </c>
-      <c r="I15" s="23" t="n">
+      <c r="I15" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="J15" s="23" t="n">
+      <c r="J15" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="K15" s="21" t="inlineStr"/>
-      <c r="L15" s="22" t="n">
+      <c r="K15" s="20" t="n">
+        <v>12938</v>
+      </c>
+      <c r="L15" s="21" t="n">
         <v>0.08</v>
       </c>
-      <c r="M15" s="23" t="n">
+      <c r="M15" s="20" t="n">
         <v>1034.7</v>
       </c>
-      <c r="N15" s="23" t="n">
+      <c r="N15" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="O15" s="23" t="n">
+      <c r="O15" s="20" t="n">
         <v>1157</v>
       </c>
-      <c r="P15" s="23" t="n">
+      <c r="P15" s="20" t="n">
         <v>47</v>
       </c>
-      <c r="Q15" s="29" t="n">
+      <c r="Q15" s="27" t="n">
         <v>-66</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  Kinh doanh bán buôn</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr"/>
-      <c r="D16" s="23" t="n">
+      <c r="C16" s="19" t="inlineStr"/>
+      <c r="D16" s="20" t="n">
         <v>4792</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="21" t="n">
         <v>0.1</v>
       </c>
-      <c r="F16" s="23" t="n">
+      <c r="F16" s="20" t="n">
         <v>473.1</v>
       </c>
-      <c r="G16" s="23" t="n">
+      <c r="G16" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="H16" s="23" t="n">
+      <c r="H16" s="20" t="n">
         <v>311</v>
       </c>
-      <c r="I16" s="23" t="n">
+      <c r="I16" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="J16" s="23" t="n">
+      <c r="J16" s="20" t="n">
         <v>178</v>
       </c>
-      <c r="K16" s="21" t="inlineStr"/>
-      <c r="L16" s="22" t="n">
+      <c r="K16" s="20" t="n">
+        <v>35000</v>
+      </c>
+      <c r="L16" s="21" t="n">
         <v>0.09</v>
       </c>
-      <c r="M16" s="23" t="n">
+      <c r="M16" s="20" t="n">
         <v>2275.1</v>
       </c>
-      <c r="N16" s="23" t="n">
+      <c r="N16" s="20" t="n">
         <v>271</v>
       </c>
-      <c r="O16" s="23" t="n">
+      <c r="O16" s="20" t="n">
         <v>2438</v>
       </c>
-      <c r="P16" s="23" t="n">
+      <c r="P16" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="Q16" s="23" t="n">
+      <c r="Q16" s="20" t="n">
         <v>119</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  Dự án</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr"/>
-      <c r="D17" s="23" t="n">
+      <c r="C17" s="19" t="inlineStr"/>
+      <c r="D17" s="20" t="n">
         <v>295</v>
       </c>
-      <c r="E17" s="22" t="n">
+      <c r="E17" s="21" t="n">
         <v>0.19</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="20" t="n">
         <v>56.1</v>
       </c>
-      <c r="G17" s="21" t="inlineStr"/>
-      <c r="H17" s="23" t="n">
+      <c r="G17" s="19" t="inlineStr"/>
+      <c r="H17" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="I17" s="21" t="inlineStr"/>
-      <c r="J17" s="29" t="n">
+      <c r="I17" s="19" t="inlineStr"/>
+      <c r="J17" s="27" t="n">
         <v>-10</v>
       </c>
-      <c r="K17" s="21" t="inlineStr"/>
-      <c r="L17" s="22" t="n">
+      <c r="K17" s="20" t="n">
+        <v>2500</v>
+      </c>
+      <c r="L17" s="21" t="n">
         <v>0.41</v>
       </c>
-      <c r="M17" s="21" t="inlineStr"/>
-      <c r="N17" s="21" t="inlineStr"/>
-      <c r="O17" s="23" t="n">
+      <c r="M17" s="20" t="n">
+        <v>1025</v>
+      </c>
+      <c r="N17" s="19" t="inlineStr"/>
+      <c r="O17" s="20" t="n">
         <v>3342</v>
       </c>
-      <c r="P17" s="21" t="inlineStr"/>
-      <c r="Q17" s="23" t="n">
+      <c r="P17" s="19" t="inlineStr"/>
+      <c r="Q17" s="20" t="n">
         <v>2038</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Việt</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr"/>
-      <c r="D18" s="17" t="inlineStr"/>
-      <c r="E18" s="18" t="n">
+      <c r="C18" s="15" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>6848</v>
+      </c>
+      <c r="E18" s="16" t="n">
         <v>0.203</v>
       </c>
-      <c r="F18" s="16" t="n">
+      <c r="F18" s="15" t="n">
         <v>1390</v>
       </c>
-      <c r="G18" s="16" t="n">
+      <c r="G18" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="16" t="n">
+      <c r="H18" s="15" t="n">
         <v>983</v>
       </c>
-      <c r="I18" s="17" t="inlineStr"/>
-      <c r="J18" s="16" t="n">
+      <c r="I18" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="J18" s="15" t="n">
         <v>382</v>
       </c>
-      <c r="K18" s="17" t="inlineStr"/>
-      <c r="L18" s="18" t="n">
+      <c r="K18" s="15" t="n">
+        <v>40294</v>
+      </c>
+      <c r="L18" s="16" t="n">
         <v>0.21</v>
       </c>
-      <c r="M18" s="16" t="n">
+      <c r="M18" s="15" t="n">
         <v>8562</v>
       </c>
-      <c r="N18" s="17" t="inlineStr"/>
-      <c r="O18" s="16" t="n">
+      <c r="N18" s="28" t="inlineStr"/>
+      <c r="O18" s="15" t="n">
         <v>6903</v>
       </c>
-      <c r="P18" s="16" t="n">
+      <c r="P18" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="Q18" s="16" t="n">
+      <c r="Q18" s="15" t="n">
         <v>1672</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Thuê máy</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr"/>
-      <c r="D19" s="27" t="n">
+      <c r="C19" s="24" t="inlineStr"/>
+      <c r="D19" s="25" t="n">
         <v>1565</v>
       </c>
-      <c r="E19" s="28" t="n">
+      <c r="E19" s="26" t="n">
         <v>0.59</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="25" t="n">
         <v>924</v>
       </c>
-      <c r="G19" s="26" t="inlineStr"/>
-      <c r="H19" s="27" t="n">
+      <c r="G19" s="24" t="inlineStr"/>
+      <c r="H19" s="25" t="n">
         <v>653</v>
       </c>
-      <c r="I19" s="26" t="inlineStr"/>
-      <c r="J19" s="27" t="n">
+      <c r="I19" s="24" t="inlineStr"/>
+      <c r="J19" s="25" t="n">
         <v>271</v>
       </c>
-      <c r="K19" s="27" t="n">
+      <c r="K19" s="25" t="n">
         <v>10876</v>
       </c>
-      <c r="L19" s="28" t="n">
+      <c r="L19" s="26" t="n">
         <v>0.58</v>
       </c>
-      <c r="M19" s="27" t="n">
+      <c r="M19" s="25" t="n">
         <v>6285</v>
       </c>
-      <c r="N19" s="26" t="inlineStr"/>
-      <c r="O19" s="27" t="n">
+      <c r="N19" s="24" t="inlineStr"/>
+      <c r="O19" s="25" t="n">
         <v>4513</v>
       </c>
-      <c r="P19" s="27" t="n">
+      <c r="P19" s="25" t="n">
         <v>11.4</v>
       </c>
-      <c r="Q19" s="27" t="n">
+      <c r="Q19" s="25" t="n">
         <v>1783</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B20" s="25" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    KDTH</t>
         </is>
       </c>
-      <c r="C20" s="26" t="inlineStr"/>
-      <c r="D20" s="27" t="n">
+      <c r="C20" s="24" t="inlineStr"/>
+      <c r="D20" s="25" t="n">
         <v>1991</v>
       </c>
-      <c r="E20" s="28" t="n">
+      <c r="E20" s="26" t="n">
         <v>0.08</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="25" t="n">
         <v>151</v>
       </c>
-      <c r="G20" s="26" t="inlineStr"/>
-      <c r="H20" s="27" t="n">
+      <c r="G20" s="24" t="inlineStr"/>
+      <c r="H20" s="25" t="n">
         <v>144</v>
       </c>
-      <c r="I20" s="27" t="n">
+      <c r="I20" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="J20" s="27" t="n">
+      <c r="J20" s="25" t="n">
         <v>14</v>
       </c>
-      <c r="K20" s="27" t="n">
+      <c r="K20" s="25" t="n">
         <v>12624</v>
       </c>
-      <c r="L20" s="28" t="n">
+      <c r="L20" s="26" t="n">
         <v>0.08</v>
       </c>
-      <c r="M20" s="27" t="n">
+      <c r="M20" s="25" t="n">
         <v>970</v>
       </c>
-      <c r="N20" s="26" t="inlineStr"/>
-      <c r="O20" s="27" t="n">
+      <c r="N20" s="24" t="inlineStr"/>
+      <c r="O20" s="25" t="n">
         <v>1022</v>
       </c>
-      <c r="P20" s="27" t="n">
+      <c r="P20" s="25" t="n">
         <v>1.5</v>
       </c>
-      <c r="Q20" s="29" t="n">
+      <c r="Q20" s="27" t="n">
         <v>-51</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B21" s="25" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    KD online</t>
         </is>
       </c>
-      <c r="C21" s="26" t="inlineStr"/>
-      <c r="D21" s="27" t="n">
+      <c r="C21" s="24" t="inlineStr"/>
+      <c r="D21" s="25" t="n">
         <v>3135</v>
       </c>
-      <c r="E21" s="28" t="n">
+      <c r="E21" s="26" t="n">
         <v>0.067</v>
       </c>
-      <c r="F21" s="27" t="n">
+      <c r="F21" s="25" t="n">
         <v>211</v>
       </c>
-      <c r="G21" s="26" t="inlineStr"/>
-      <c r="H21" s="27" t="n">
+      <c r="G21" s="24" t="inlineStr"/>
+      <c r="H21" s="25" t="n">
         <v>149</v>
       </c>
-      <c r="I21" s="26" t="inlineStr"/>
-      <c r="J21" s="27" t="n">
+      <c r="I21" s="24" t="inlineStr"/>
+      <c r="J21" s="25" t="n">
         <v>62</v>
       </c>
-      <c r="K21" s="27" t="n">
+      <c r="K21" s="25" t="n">
         <v>16138</v>
       </c>
-      <c r="L21" s="28" t="n">
+      <c r="L21" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="M21" s="27" t="n">
+      <c r="M21" s="25" t="n">
         <v>998</v>
       </c>
-      <c r="N21" s="26" t="inlineStr"/>
-      <c r="O21" s="27" t="n">
+      <c r="N21" s="24" t="inlineStr"/>
+      <c r="O21" s="25" t="n">
         <v>1116</v>
       </c>
-      <c r="P21" s="27" t="n">
+      <c r="P21" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="Q21" s="29" t="n">
+      <c r="Q21" s="27" t="n">
         <v>-118</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B22" s="25" t="inlineStr">
+      <c r="B22" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Cửa hàng</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr"/>
-      <c r="D22" s="27" t="n">
+      <c r="C22" s="24" t="inlineStr"/>
+      <c r="D22" s="25" t="n">
         <v>157</v>
       </c>
-      <c r="E22" s="28" t="n">
+      <c r="E22" s="26" t="n">
         <v>0.499</v>
       </c>
-      <c r="F22" s="27" t="n">
+      <c r="F22" s="25" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="G22" s="26" t="inlineStr"/>
-      <c r="H22" s="27" t="n">
+      <c r="G22" s="24" t="inlineStr"/>
+      <c r="H22" s="25" t="n">
         <v>37</v>
       </c>
-      <c r="I22" s="26" t="inlineStr"/>
-      <c r="J22" s="27" t="n">
+      <c r="I22" s="24" t="inlineStr"/>
+      <c r="J22" s="25" t="n">
         <v>42</v>
       </c>
-      <c r="K22" s="27" t="n">
+      <c r="K22" s="25" t="n">
         <v>656</v>
       </c>
-      <c r="L22" s="28" t="n">
+      <c r="L22" s="26" t="n">
         <v>0.47</v>
       </c>
-      <c r="M22" s="27" t="n">
+      <c r="M22" s="25" t="n">
         <v>310</v>
       </c>
-      <c r="N22" s="26" t="inlineStr"/>
-      <c r="O22" s="27" t="n">
+      <c r="N22" s="24" t="inlineStr"/>
+      <c r="O22" s="25" t="n">
         <v>252</v>
       </c>
-      <c r="P22" s="26" t="inlineStr"/>
-      <c r="Q22" s="27" t="n">
+      <c r="P22" s="24" t="inlineStr"/>
+      <c r="Q22" s="25" t="n">
         <v>58</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>ITSS</t>
         </is>
       </c>
-      <c r="C23" s="16" t="n">
+      <c r="C23" s="15" t="n">
         <v>5000</v>
       </c>
-      <c r="D23" s="16" t="n">
+      <c r="D23" s="15" t="n">
         <v>524</v>
       </c>
-      <c r="E23" s="18" t="n">
+      <c r="E23" s="16" t="n">
         <v>0.374</v>
       </c>
-      <c r="F23" s="16" t="n">
+      <c r="F23" s="15" t="n">
         <v>196</v>
       </c>
-      <c r="G23" s="17" t="inlineStr"/>
-      <c r="H23" s="16" t="n">
+      <c r="G23" s="28" t="inlineStr"/>
+      <c r="H23" s="15" t="n">
         <v>87</v>
       </c>
-      <c r="I23" s="16" t="n">
+      <c r="I23" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="J23" s="16" t="n">
+      <c r="J23" s="15" t="n">
         <v>113</v>
       </c>
-      <c r="K23" s="16" t="n">
+      <c r="K23" s="15" t="n">
         <v>2915</v>
       </c>
-      <c r="L23" s="18" t="n">
+      <c r="L23" s="16" t="n">
         <v>0.35</v>
       </c>
-      <c r="M23" s="16" t="n">
+      <c r="M23" s="15" t="n">
         <v>1028</v>
       </c>
-      <c r="N23" s="17" t="inlineStr"/>
-      <c r="O23" s="16" t="n">
+      <c r="N23" s="28" t="inlineStr"/>
+      <c r="O23" s="15" t="n">
         <v>859</v>
       </c>
-      <c r="P23" s="30" t="n">
+      <c r="P23" s="29" t="n">
         <v>-4</v>
       </c>
-      <c r="Q23" s="16" t="n">
+      <c r="Q23" s="15" t="n">
         <v>165</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>CTY VPS</t>
         </is>
       </c>
-      <c r="C24" s="16" t="n">
+      <c r="C24" s="15" t="n">
         <v>10000</v>
       </c>
-      <c r="D24" s="17" t="inlineStr"/>
-      <c r="E24" s="18" t="n">
+      <c r="D24" s="15" t="n">
+        <v>14951</v>
+      </c>
+      <c r="E24" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="17" t="inlineStr"/>
-      <c r="G24" s="17" t="inlineStr"/>
-      <c r="H24" s="17" t="inlineStr"/>
-      <c r="I24" s="17" t="inlineStr"/>
-      <c r="J24" s="30" t="n">
+      <c r="F24" s="28" t="inlineStr"/>
+      <c r="G24" s="28" t="inlineStr"/>
+      <c r="H24" s="15" t="n">
+        <v>2327</v>
+      </c>
+      <c r="I24" s="15" t="n">
+        <v>1033</v>
+      </c>
+      <c r="J24" s="29" t="n">
         <v>-828</v>
       </c>
-      <c r="K24" s="17" t="inlineStr"/>
-      <c r="L24" s="17" t="inlineStr"/>
-      <c r="M24" s="17" t="inlineStr"/>
-      <c r="N24" s="17" t="inlineStr"/>
-      <c r="O24" s="17" t="inlineStr"/>
-      <c r="P24" s="16" t="n">
+      <c r="K24" s="15" t="n">
+        <v>16633</v>
+      </c>
+      <c r="L24" s="28" t="inlineStr"/>
+      <c r="M24" s="15" t="n">
+        <v>2288</v>
+      </c>
+      <c r="N24" s="28" t="inlineStr"/>
+      <c r="O24" s="15" t="n">
+        <v>14400</v>
+      </c>
+      <c r="P24" s="15" t="n">
         <v>7665</v>
       </c>
-      <c r="Q24" s="30" t="n">
+      <c r="Q24" s="29" t="n">
         <v>-4447</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    VP VPS - hoạt động KD</t>
         </is>
       </c>
-      <c r="C25" s="26" t="inlineStr"/>
-      <c r="D25" s="27" t="n">
+      <c r="C25" s="24" t="inlineStr"/>
+      <c r="D25" s="25" t="n">
         <v>14951</v>
       </c>
-      <c r="E25" s="28" t="n">
+      <c r="E25" s="26" t="n">
         <v>0.031</v>
       </c>
-      <c r="F25" s="27" t="n">
+      <c r="F25" s="25" t="n">
         <v>466</v>
       </c>
-      <c r="G25" s="26" t="inlineStr"/>
-      <c r="H25" s="27" t="n">
+      <c r="G25" s="24" t="inlineStr"/>
+      <c r="H25" s="25" t="n">
         <v>748</v>
       </c>
-      <c r="I25" s="27" t="n">
+      <c r="I25" s="25" t="n">
         <v>419</v>
       </c>
-      <c r="J25" s="27" t="n">
+      <c r="J25" s="25" t="n">
         <v>137</v>
       </c>
-      <c r="K25" s="27" t="n">
+      <c r="K25" s="25" t="n">
         <v>16633</v>
       </c>
-      <c r="L25" s="28" t="n">
+      <c r="L25" s="26" t="n">
         <v>0.14</v>
       </c>
-      <c r="M25" s="27" t="n">
+      <c r="M25" s="25" t="n">
         <v>2288</v>
       </c>
-      <c r="N25" s="26" t="inlineStr"/>
-      <c r="O25" s="27" t="n">
+      <c r="N25" s="24" t="inlineStr"/>
+      <c r="O25" s="25" t="n">
         <v>4673</v>
       </c>
-      <c r="P25" s="27" t="n">
+      <c r="P25" s="25" t="n">
         <v>2732</v>
       </c>
-      <c r="Q25" s="27" t="n">
+      <c r="Q25" s="25" t="n">
         <v>347</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B26" s="25" t="inlineStr">
+      <c r="B26" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    HĐ đầu tư Tài chính</t>
         </is>
       </c>
-      <c r="C26" s="26" t="inlineStr"/>
-      <c r="D26" s="27" t="n">
+      <c r="C26" s="24" t="inlineStr"/>
+      <c r="D26" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="28" t="n">
+      <c r="E26" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="27" t="n">
+      <c r="F26" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="26" t="inlineStr"/>
-      <c r="H26" s="27" t="n">
+      <c r="G26" s="24" t="inlineStr"/>
+      <c r="H26" s="25" t="n">
         <v>1579</v>
       </c>
-      <c r="I26" s="27" t="n">
+      <c r="I26" s="25" t="n">
         <v>614</v>
       </c>
-      <c r="J26" s="29" t="n">
+      <c r="J26" s="27" t="n">
         <v>-965</v>
       </c>
-      <c r="K26" s="27" t="n">
+      <c r="K26" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="L26" s="28" t="n">
+      <c r="L26" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="M26" s="27" t="n">
+      <c r="M26" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="N26" s="26" t="inlineStr"/>
-      <c r="O26" s="27" t="n">
+      <c r="N26" s="24" t="inlineStr"/>
+      <c r="O26" s="25" t="n">
         <v>9727</v>
       </c>
-      <c r="P26" s="27" t="n">
+      <c r="P26" s="25" t="n">
         <v>4933</v>
       </c>
-      <c r="Q26" s="29" t="n">
+      <c r="Q26" s="27" t="n">
         <v>-4794</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>XESCO (Xem Sơn)</t>
         </is>
       </c>
-      <c r="C27" s="16" t="n">
+      <c r="C27" s="15" t="n">
         <v>15000</v>
       </c>
-      <c r="D27" s="17" t="inlineStr"/>
-      <c r="E27" s="18" t="n">
+      <c r="D27" s="15" t="n">
+        <v>10326</v>
+      </c>
+      <c r="E27" s="16" t="n">
         <v>0.28</v>
       </c>
-      <c r="F27" s="16" t="n">
+      <c r="F27" s="15" t="n">
         <v>2912</v>
       </c>
-      <c r="G27" s="17" t="inlineStr"/>
-      <c r="H27" s="16" t="n">
+      <c r="G27" s="28" t="inlineStr"/>
+      <c r="H27" s="15" t="n">
         <v>2129</v>
       </c>
-      <c r="I27" s="16" t="n">
+      <c r="I27" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J27" s="16" t="n">
+      <c r="J27" s="15" t="n">
         <v>834</v>
       </c>
-      <c r="K27" s="17" t="inlineStr"/>
-      <c r="L27" s="18" t="n">
+      <c r="K27" s="15" t="n">
+        <v>69425</v>
+      </c>
+      <c r="L27" s="16" t="n">
         <v>0.27</v>
       </c>
-      <c r="M27" s="16" t="n">
+      <c r="M27" s="15" t="n">
         <v>18667</v>
       </c>
-      <c r="N27" s="17" t="inlineStr"/>
-      <c r="O27" s="16" t="n">
+      <c r="N27" s="28" t="inlineStr"/>
+      <c r="O27" s="15" t="n">
         <v>14626</v>
       </c>
-      <c r="P27" s="16" t="n">
+      <c r="P27" s="15" t="n">
         <v>226</v>
       </c>
-      <c r="Q27" s="16" t="n">
+      <c r="Q27" s="15" t="n">
         <v>4267</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  Xesco - KD</t>
         </is>
       </c>
-      <c r="C28" s="21" t="inlineStr"/>
-      <c r="D28" s="23" t="n">
+      <c r="C28" s="19" t="inlineStr"/>
+      <c r="D28" s="20" t="n">
         <v>7182</v>
       </c>
-      <c r="E28" s="22" t="n">
+      <c r="E28" s="21" t="n">
         <v>0.16</v>
       </c>
-      <c r="F28" s="23" t="n">
+      <c r="F28" s="20" t="n">
         <v>1168</v>
       </c>
-      <c r="G28" s="21" t="inlineStr"/>
-      <c r="H28" s="23" t="n">
+      <c r="G28" s="19" t="inlineStr"/>
+      <c r="H28" s="20" t="n">
         <v>850</v>
       </c>
-      <c r="I28" s="21" t="inlineStr"/>
-      <c r="J28" s="23" t="n">
+      <c r="I28" s="19" t="inlineStr"/>
+      <c r="J28" s="20" t="n">
         <v>318</v>
       </c>
-      <c r="K28" s="23" t="n">
+      <c r="K28" s="20" t="n">
         <v>48562</v>
       </c>
-      <c r="L28" s="22" t="n">
+      <c r="L28" s="21" t="n">
         <v>0.15</v>
       </c>
-      <c r="M28" s="23" t="n">
+      <c r="M28" s="20" t="n">
         <v>7129</v>
       </c>
-      <c r="N28" s="21" t="inlineStr"/>
-      <c r="O28" s="23" t="n">
+      <c r="N28" s="19" t="inlineStr"/>
+      <c r="O28" s="20" t="n">
         <v>5542</v>
       </c>
-      <c r="P28" s="23" t="n">
+      <c r="P28" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="Q28" s="23" t="n">
+      <c r="Q28" s="20" t="n">
         <v>1687</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="24" t="inlineStr"/>
-      <c r="B29" s="25" t="inlineStr">
+      <c r="A29" s="22" t="inlineStr"/>
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Bán máy lẻ</t>
         </is>
       </c>
-      <c r="C29" s="26" t="inlineStr"/>
-      <c r="D29" s="27" t="n">
+      <c r="C29" s="24" t="inlineStr"/>
+      <c r="D29" s="25" t="n">
         <v>191</v>
       </c>
-      <c r="E29" s="28" t="n">
+      <c r="E29" s="26" t="n">
         <v>0.26</v>
       </c>
-      <c r="F29" s="27" t="n">
+      <c r="F29" s="25" t="n">
         <v>49</v>
       </c>
-      <c r="G29" s="26" t="inlineStr"/>
-      <c r="H29" s="27" t="n">
+      <c r="G29" s="24" t="inlineStr"/>
+      <c r="H29" s="25" t="n">
         <v>71</v>
       </c>
-      <c r="I29" s="26" t="inlineStr"/>
-      <c r="J29" s="29" t="n">
+      <c r="I29" s="24" t="inlineStr"/>
+      <c r="J29" s="27" t="n">
         <v>-22</v>
       </c>
-      <c r="K29" s="27" t="n">
+      <c r="K29" s="25" t="n">
         <v>3397</v>
       </c>
-      <c r="L29" s="28" t="n">
+      <c r="L29" s="26" t="n">
         <v>0.23</v>
       </c>
-      <c r="M29" s="27" t="n">
+      <c r="M29" s="25" t="n">
         <v>777</v>
       </c>
-      <c r="N29" s="26" t="inlineStr"/>
-      <c r="O29" s="27" t="n">
+      <c r="N29" s="24" t="inlineStr"/>
+      <c r="O29" s="25" t="n">
         <v>601</v>
       </c>
-      <c r="P29" s="26" t="inlineStr"/>
-      <c r="Q29" s="27" t="n">
+      <c r="P29" s="24" t="inlineStr"/>
+      <c r="Q29" s="25" t="n">
         <v>176</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="24" t="inlineStr"/>
-      <c r="B30" s="25" t="inlineStr">
+      <c r="A30" s="22" t="inlineStr"/>
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    KD sỉ</t>
         </is>
       </c>
-      <c r="C30" s="26" t="inlineStr"/>
-      <c r="D30" s="27" t="n">
+      <c r="C30" s="24" t="inlineStr"/>
+      <c r="D30" s="25" t="n">
         <v>4032</v>
       </c>
-      <c r="E30" s="28" t="n">
+      <c r="E30" s="26" t="n">
         <v>0.17</v>
       </c>
-      <c r="F30" s="27" t="n">
+      <c r="F30" s="25" t="n">
         <v>690</v>
       </c>
-      <c r="G30" s="26" t="inlineStr"/>
-      <c r="H30" s="27" t="n">
+      <c r="G30" s="24" t="inlineStr"/>
+      <c r="H30" s="25" t="n">
         <v>479</v>
       </c>
-      <c r="I30" s="26" t="inlineStr"/>
-      <c r="J30" s="27" t="n">
+      <c r="I30" s="24" t="inlineStr"/>
+      <c r="J30" s="25" t="n">
         <v>211</v>
       </c>
-      <c r="K30" s="27" t="n">
+      <c r="K30" s="25" t="n">
         <v>22834</v>
       </c>
-      <c r="L30" s="28" t="n">
+      <c r="L30" s="26" t="n">
         <v>0.16</v>
       </c>
-      <c r="M30" s="27" t="n">
+      <c r="M30" s="25" t="n">
         <v>3727</v>
       </c>
-      <c r="N30" s="26" t="inlineStr"/>
-      <c r="O30" s="27" t="n">
+      <c r="N30" s="24" t="inlineStr"/>
+      <c r="O30" s="25" t="n">
         <v>3151</v>
       </c>
-      <c r="P30" s="27" t="n">
+      <c r="P30" s="25" t="n">
         <v>100</v>
       </c>
-      <c r="Q30" s="27" t="n">
+      <c r="Q30" s="25" t="n">
         <v>676</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="24" t="inlineStr"/>
-      <c r="B31" s="25" t="inlineStr">
+      <c r="A31" s="22" t="inlineStr"/>
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    KD Online</t>
         </is>
       </c>
-      <c r="C31" s="26" t="inlineStr"/>
-      <c r="D31" s="27" t="n">
+      <c r="C31" s="24" t="inlineStr"/>
+      <c r="D31" s="25" t="n">
         <v>2539</v>
       </c>
-      <c r="E31" s="28" t="n">
+      <c r="E31" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F31" s="27" t="n">
+      <c r="F31" s="25" t="n">
         <v>135</v>
       </c>
-      <c r="G31" s="26" t="inlineStr"/>
-      <c r="H31" s="27" t="n">
+      <c r="G31" s="24" t="inlineStr"/>
+      <c r="H31" s="25" t="n">
         <v>129</v>
       </c>
-      <c r="I31" s="26" t="inlineStr"/>
-      <c r="J31" s="27" t="n">
+      <c r="I31" s="24" t="inlineStr"/>
+      <c r="J31" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="K31" s="27" t="n">
+      <c r="K31" s="25" t="n">
         <v>19679</v>
       </c>
-      <c r="L31" s="28" t="n">
+      <c r="L31" s="26" t="n">
         <v>0.04</v>
       </c>
-      <c r="M31" s="27" t="n">
+      <c r="M31" s="25" t="n">
         <v>769</v>
       </c>
-      <c r="N31" s="26" t="inlineStr"/>
-      <c r="O31" s="27" t="n">
+      <c r="N31" s="24" t="inlineStr"/>
+      <c r="O31" s="25" t="n">
         <v>741</v>
       </c>
-      <c r="P31" s="26" t="inlineStr"/>
-      <c r="Q31" s="27" t="n">
+      <c r="P31" s="24" t="inlineStr"/>
+      <c r="Q31" s="25" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="24" t="inlineStr"/>
-      <c r="B32" s="25" t="inlineStr">
+      <c r="A32" s="22" t="inlineStr"/>
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    KD Thuê máy</t>
         </is>
       </c>
-      <c r="C32" s="26" t="inlineStr"/>
-      <c r="D32" s="27" t="n">
+      <c r="C32" s="24" t="inlineStr"/>
+      <c r="D32" s="25" t="n">
         <v>420</v>
       </c>
-      <c r="E32" s="28" t="n">
+      <c r="E32" s="26" t="n">
         <v>0.7</v>
       </c>
-      <c r="F32" s="27" t="n">
+      <c r="F32" s="25" t="n">
         <v>294</v>
       </c>
-      <c r="G32" s="26" t="inlineStr"/>
-      <c r="H32" s="27" t="n">
+      <c r="G32" s="24" t="inlineStr"/>
+      <c r="H32" s="25" t="n">
         <v>171</v>
       </c>
-      <c r="I32" s="26" t="inlineStr"/>
-      <c r="J32" s="27" t="n">
+      <c r="I32" s="24" t="inlineStr"/>
+      <c r="J32" s="25" t="n">
         <v>123</v>
       </c>
-      <c r="K32" s="27" t="n">
+      <c r="K32" s="25" t="n">
         <v>2653</v>
       </c>
-      <c r="L32" s="28" t="n">
+      <c r="L32" s="26" t="n">
         <v>0.7</v>
       </c>
-      <c r="M32" s="27" t="n">
+      <c r="M32" s="25" t="n">
         <v>1856</v>
       </c>
-      <c r="N32" s="26" t="inlineStr"/>
-      <c r="O32" s="27" t="n">
+      <c r="N32" s="24" t="inlineStr"/>
+      <c r="O32" s="25" t="n">
         <v>1049</v>
       </c>
-      <c r="P32" s="26" t="inlineStr"/>
-      <c r="Q32" s="27" t="n">
+      <c r="P32" s="24" t="inlineStr"/>
+      <c r="Q32" s="25" t="n">
         <v>807</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">  Xesco - KT</t>
         </is>
       </c>
-      <c r="C33" s="21" t="inlineStr"/>
-      <c r="D33" s="23" t="n">
+      <c r="C33" s="19" t="inlineStr"/>
+      <c r="D33" s="20" t="n">
         <v>3144</v>
       </c>
-      <c r="E33" s="22" t="n">
+      <c r="E33" s="21" t="n">
         <v>0.55</v>
       </c>
-      <c r="F33" s="23" t="n">
+      <c r="F33" s="20" t="n">
         <v>1744</v>
       </c>
-      <c r="G33" s="21" t="inlineStr"/>
-      <c r="H33" s="23" t="n">
+      <c r="G33" s="19" t="inlineStr"/>
+      <c r="H33" s="20" t="n">
         <v>1279</v>
       </c>
-      <c r="I33" s="21" t="inlineStr"/>
-      <c r="J33" s="23" t="n">
+      <c r="I33" s="19" t="inlineStr"/>
+      <c r="J33" s="20" t="n">
         <v>465</v>
       </c>
-      <c r="K33" s="23" t="n">
+      <c r="K33" s="20" t="n">
         <v>20863</v>
       </c>
-      <c r="L33" s="22" t="n">
+      <c r="L33" s="21" t="n">
         <v>0.55</v>
       </c>
-      <c r="M33" s="23" t="n">
+      <c r="M33" s="20" t="n">
         <v>11538</v>
       </c>
-      <c r="N33" s="21" t="inlineStr"/>
-      <c r="O33" s="23" t="n">
+      <c r="N33" s="19" t="inlineStr"/>
+      <c r="O33" s="20" t="n">
         <v>9084</v>
       </c>
-      <c r="P33" s="23" t="n">
+      <c r="P33" s="20" t="n">
         <v>126</v>
       </c>
-      <c r="Q33" s="23" t="n">
+      <c r="Q33" s="20" t="n">
         <v>2580</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr"/>
-      <c r="B34" s="25" t="inlineStr">
+      <c r="A34" s="22" t="inlineStr"/>
+      <c r="B34" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Thuê máy</t>
         </is>
       </c>
-      <c r="C34" s="26" t="inlineStr"/>
-      <c r="D34" s="27" t="n">
+      <c r="C34" s="24" t="inlineStr"/>
+      <c r="D34" s="25" t="n">
         <v>1502</v>
       </c>
-      <c r="E34" s="28" t="n">
+      <c r="E34" s="26" t="n">
         <v>0.66</v>
       </c>
-      <c r="F34" s="27" t="n">
+      <c r="F34" s="25" t="n">
         <v>994</v>
       </c>
-      <c r="G34" s="26" t="inlineStr"/>
-      <c r="H34" s="27" t="n">
+      <c r="G34" s="24" t="inlineStr"/>
+      <c r="H34" s="25" t="n">
         <v>776</v>
       </c>
-      <c r="I34" s="26" t="inlineStr"/>
-      <c r="J34" s="27" t="n">
+      <c r="I34" s="24" t="inlineStr"/>
+      <c r="J34" s="25" t="n">
         <v>218</v>
       </c>
-      <c r="K34" s="27" t="n">
+      <c r="K34" s="25" t="n">
         <v>10358</v>
       </c>
-      <c r="L34" s="28" t="n">
+      <c r="L34" s="26" t="n">
         <v>0.67</v>
       </c>
-      <c r="M34" s="27" t="n">
+      <c r="M34" s="25" t="n">
         <v>6958</v>
       </c>
-      <c r="N34" s="26" t="inlineStr"/>
-      <c r="O34" s="27" t="n">
+      <c r="N34" s="24" t="inlineStr"/>
+      <c r="O34" s="25" t="n">
         <v>5723</v>
       </c>
-      <c r="P34" s="27" t="n">
+      <c r="P34" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="Q34" s="27" t="n">
+      <c r="Q34" s="25" t="n">
         <v>1241</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="24" t="inlineStr"/>
-      <c r="B35" s="25" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr"/>
+      <c r="B35" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Metercharge</t>
         </is>
       </c>
-      <c r="C35" s="26" t="inlineStr"/>
-      <c r="D35" s="27" t="n">
+      <c r="C35" s="24" t="inlineStr"/>
+      <c r="D35" s="25" t="n">
         <v>278</v>
       </c>
-      <c r="E35" s="28" t="n">
+      <c r="E35" s="26" t="n">
         <v>0.59</v>
       </c>
-      <c r="F35" s="27" t="n">
+      <c r="F35" s="25" t="n">
         <v>164</v>
       </c>
-      <c r="G35" s="26" t="inlineStr"/>
-      <c r="H35" s="26" t="inlineStr"/>
-      <c r="I35" s="26" t="inlineStr"/>
-      <c r="J35" s="27" t="n">
+      <c r="G35" s="24" t="inlineStr"/>
+      <c r="H35" s="24" t="inlineStr"/>
+      <c r="I35" s="24" t="inlineStr"/>
+      <c r="J35" s="25" t="n">
         <v>164</v>
       </c>
-      <c r="K35" s="27" t="n">
+      <c r="K35" s="25" t="n">
         <v>1869</v>
       </c>
-      <c r="L35" s="28" t="n">
+      <c r="L35" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="M35" s="27" t="n">
+      <c r="M35" s="25" t="n">
         <v>1114</v>
       </c>
-      <c r="N35" s="26" t="inlineStr"/>
-      <c r="O35" s="26" t="inlineStr"/>
-      <c r="P35" s="26" t="inlineStr"/>
-      <c r="Q35" s="27" t="n">
+      <c r="N35" s="24" t="inlineStr"/>
+      <c r="O35" s="24" t="inlineStr"/>
+      <c r="P35" s="24" t="inlineStr"/>
+      <c r="Q35" s="25" t="n">
         <v>1114</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="24" t="inlineStr"/>
-      <c r="B36" s="25" t="inlineStr">
+      <c r="A36" s="22" t="inlineStr"/>
+      <c r="B36" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Dịch vụ</t>
         </is>
       </c>
-      <c r="C36" s="26" t="inlineStr"/>
-      <c r="D36" s="27" t="n">
+      <c r="C36" s="24" t="inlineStr"/>
+      <c r="D36" s="25" t="n">
         <v>1364</v>
       </c>
-      <c r="E36" s="28" t="n">
+      <c r="E36" s="26" t="n">
         <v>0.43</v>
       </c>
-      <c r="F36" s="27" t="n">
+      <c r="F36" s="25" t="n">
         <v>586</v>
       </c>
-      <c r="G36" s="26" t="inlineStr"/>
-      <c r="H36" s="27" t="n">
+      <c r="G36" s="24" t="inlineStr"/>
+      <c r="H36" s="25" t="n">
         <v>503</v>
       </c>
-      <c r="I36" s="26" t="inlineStr"/>
-      <c r="J36" s="27" t="n">
+      <c r="I36" s="24" t="inlineStr"/>
+      <c r="J36" s="25" t="n">
         <v>83</v>
       </c>
-      <c r="K36" s="27" t="n">
+      <c r="K36" s="25" t="n">
         <v>8636</v>
       </c>
-      <c r="L36" s="28" t="n">
+      <c r="L36" s="26" t="n">
         <v>0.4</v>
       </c>
-      <c r="M36" s="27" t="n">
+      <c r="M36" s="25" t="n">
         <v>3466</v>
       </c>
-      <c r="N36" s="26" t="inlineStr"/>
-      <c r="O36" s="27" t="n">
+      <c r="N36" s="24" t="inlineStr"/>
+      <c r="O36" s="25" t="n">
         <v>3361</v>
       </c>
-      <c r="P36" s="27" t="n">
+      <c r="P36" s="25" t="n">
         <v>120</v>
       </c>
-      <c r="Q36" s="27" t="n">
+      <c r="Q36" s="25" t="n">
         <v>225</v>
       </c>
     </row>
@@ -2171,13 +2230,13 @@
       <c r="D37" s="10" t="n">
         <v>1674</v>
       </c>
-      <c r="E37" s="12" t="n">
+      <c r="E37" s="11" t="n">
         <v>0.14</v>
       </c>
       <c r="F37" s="10" t="n">
         <v>239</v>
       </c>
-      <c r="G37" s="11" t="inlineStr"/>
+      <c r="G37" s="30" t="inlineStr"/>
       <c r="H37" s="10" t="n">
         <v>220</v>
       </c>
@@ -2190,13 +2249,13 @@
       <c r="K37" s="10" t="n">
         <v>11251</v>
       </c>
-      <c r="L37" s="12" t="n">
+      <c r="L37" s="11" t="n">
         <v>0.2</v>
       </c>
       <c r="M37" s="10" t="n">
         <v>2267</v>
       </c>
-      <c r="N37" s="11" t="inlineStr"/>
+      <c r="N37" s="30" t="inlineStr"/>
       <c r="O37" s="10" t="n">
         <v>1515</v>
       </c>
@@ -2208,249 +2267,249 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="24" t="inlineStr"/>
-      <c r="B38" s="25" t="inlineStr">
+      <c r="A38" s="22" t="inlineStr"/>
+      <c r="B38" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Kinh doanh máy - bán buôn</t>
         </is>
       </c>
-      <c r="C38" s="26" t="inlineStr"/>
-      <c r="D38" s="27" t="n">
+      <c r="C38" s="24" t="inlineStr"/>
+      <c r="D38" s="25" t="n">
         <v>993</v>
       </c>
-      <c r="E38" s="28" t="n">
+      <c r="E38" s="26" t="n">
         <v>0.05</v>
       </c>
-      <c r="F38" s="27" t="n">
+      <c r="F38" s="25" t="n">
         <v>49</v>
       </c>
-      <c r="G38" s="26" t="inlineStr"/>
-      <c r="H38" s="26" t="inlineStr"/>
-      <c r="I38" s="26" t="inlineStr"/>
-      <c r="J38" s="26" t="inlineStr"/>
-      <c r="K38" s="27" t="n">
+      <c r="G38" s="24" t="inlineStr"/>
+      <c r="H38" s="24" t="inlineStr"/>
+      <c r="I38" s="24" t="inlineStr"/>
+      <c r="J38" s="24" t="inlineStr"/>
+      <c r="K38" s="25" t="n">
         <v>5840</v>
       </c>
-      <c r="L38" s="28" t="n">
+      <c r="L38" s="26" t="n">
         <v>0.08</v>
       </c>
-      <c r="M38" s="27" t="n">
+      <c r="M38" s="25" t="n">
         <v>496</v>
       </c>
-      <c r="N38" s="26" t="inlineStr"/>
-      <c r="O38" s="26" t="inlineStr"/>
-      <c r="P38" s="26" t="inlineStr"/>
-      <c r="Q38" s="26" t="inlineStr"/>
+      <c r="N38" s="24" t="inlineStr"/>
+      <c r="O38" s="24" t="inlineStr"/>
+      <c r="P38" s="24" t="inlineStr"/>
+      <c r="Q38" s="24" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="24" t="inlineStr"/>
-      <c r="B39" s="25" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr"/>
+      <c r="B39" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Kinh doanh linh kiện - bán buôn</t>
         </is>
       </c>
-      <c r="C39" s="26" t="inlineStr"/>
-      <c r="D39" s="27" t="n">
+      <c r="C39" s="24" t="inlineStr"/>
+      <c r="D39" s="25" t="n">
         <v>231</v>
       </c>
-      <c r="E39" s="28" t="n">
+      <c r="E39" s="26" t="n">
         <v>0.14</v>
       </c>
-      <c r="F39" s="27" t="n">
+      <c r="F39" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="G39" s="26" t="inlineStr"/>
-      <c r="H39" s="26" t="inlineStr"/>
-      <c r="I39" s="26" t="inlineStr"/>
-      <c r="J39" s="26" t="inlineStr"/>
-      <c r="K39" s="27" t="n">
+      <c r="G39" s="24" t="inlineStr"/>
+      <c r="H39" s="24" t="inlineStr"/>
+      <c r="I39" s="24" t="inlineStr"/>
+      <c r="J39" s="24" t="inlineStr"/>
+      <c r="K39" s="25" t="n">
         <v>1788</v>
       </c>
-      <c r="L39" s="28" t="n">
+      <c r="L39" s="26" t="n">
         <v>0.15</v>
       </c>
-      <c r="M39" s="27" t="n">
+      <c r="M39" s="25" t="n">
         <v>268</v>
       </c>
-      <c r="N39" s="26" t="inlineStr"/>
-      <c r="O39" s="26" t="inlineStr"/>
-      <c r="P39" s="26" t="inlineStr"/>
-      <c r="Q39" s="26" t="inlineStr"/>
+      <c r="N39" s="24" t="inlineStr"/>
+      <c r="O39" s="24" t="inlineStr"/>
+      <c r="P39" s="24" t="inlineStr"/>
+      <c r="Q39" s="24" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="24" t="inlineStr"/>
-      <c r="B40" s="25" t="inlineStr">
+      <c r="A40" s="22" t="inlineStr"/>
+      <c r="B40" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Shopee-Online</t>
         </is>
       </c>
-      <c r="C40" s="26" t="inlineStr"/>
-      <c r="D40" s="27" t="n">
+      <c r="C40" s="24" t="inlineStr"/>
+      <c r="D40" s="25" t="n">
         <v>93</v>
       </c>
-      <c r="E40" s="28" t="n">
+      <c r="E40" s="26" t="n">
         <v>0.02</v>
       </c>
-      <c r="F40" s="27" t="n">
+      <c r="F40" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="G40" s="26" t="inlineStr"/>
-      <c r="H40" s="26" t="inlineStr"/>
-      <c r="I40" s="26" t="inlineStr"/>
-      <c r="J40" s="26" t="inlineStr"/>
-      <c r="K40" s="27" t="n">
+      <c r="G40" s="24" t="inlineStr"/>
+      <c r="H40" s="24" t="inlineStr"/>
+      <c r="I40" s="24" t="inlineStr"/>
+      <c r="J40" s="24" t="inlineStr"/>
+      <c r="K40" s="25" t="n">
         <v>806</v>
       </c>
-      <c r="L40" s="28" t="n">
+      <c r="L40" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="M40" s="27" t="n">
+      <c r="M40" s="25" t="n">
         <v>45</v>
       </c>
-      <c r="N40" s="26" t="inlineStr"/>
-      <c r="O40" s="26" t="inlineStr"/>
-      <c r="P40" s="26" t="inlineStr"/>
-      <c r="Q40" s="26" t="inlineStr"/>
+      <c r="N40" s="24" t="inlineStr"/>
+      <c r="O40" s="24" t="inlineStr"/>
+      <c r="P40" s="24" t="inlineStr"/>
+      <c r="Q40" s="24" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="24" t="inlineStr"/>
-      <c r="B41" s="25" t="inlineStr">
+      <c r="A41" s="22" t="inlineStr"/>
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Dịch vụ</t>
         </is>
       </c>
-      <c r="C41" s="26" t="inlineStr"/>
-      <c r="D41" s="27" t="n">
+      <c r="C41" s="24" t="inlineStr"/>
+      <c r="D41" s="25" t="n">
         <v>225</v>
       </c>
-      <c r="E41" s="28" t="n">
+      <c r="E41" s="26" t="n">
         <v>0.43</v>
       </c>
-      <c r="F41" s="27" t="n">
+      <c r="F41" s="25" t="n">
         <v>97</v>
       </c>
-      <c r="G41" s="26" t="inlineStr"/>
-      <c r="H41" s="26" t="inlineStr"/>
-      <c r="I41" s="26" t="inlineStr"/>
-      <c r="J41" s="26" t="inlineStr"/>
-      <c r="K41" s="27" t="n">
+      <c r="G41" s="24" t="inlineStr"/>
+      <c r="H41" s="24" t="inlineStr"/>
+      <c r="I41" s="24" t="inlineStr"/>
+      <c r="J41" s="24" t="inlineStr"/>
+      <c r="K41" s="25" t="n">
         <v>1467</v>
       </c>
-      <c r="L41" s="28" t="n">
+      <c r="L41" s="26" t="n">
         <v>0.49</v>
       </c>
-      <c r="M41" s="27" t="n">
+      <c r="M41" s="25" t="n">
         <v>720</v>
       </c>
-      <c r="N41" s="26" t="inlineStr"/>
-      <c r="O41" s="26" t="inlineStr"/>
-      <c r="P41" s="26" t="inlineStr"/>
-      <c r="Q41" s="26" t="inlineStr"/>
+      <c r="N41" s="24" t="inlineStr"/>
+      <c r="O41" s="24" t="inlineStr"/>
+      <c r="P41" s="24" t="inlineStr"/>
+      <c r="Q41" s="24" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="inlineStr"/>
-      <c r="B42" s="25" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr"/>
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Thuê máy</t>
         </is>
       </c>
-      <c r="C42" s="26" t="inlineStr"/>
-      <c r="D42" s="27" t="n">
+      <c r="C42" s="24" t="inlineStr"/>
+      <c r="D42" s="25" t="n">
         <v>81</v>
       </c>
-      <c r="E42" s="28" t="n">
+      <c r="E42" s="26" t="n">
         <v>0.25</v>
       </c>
-      <c r="F42" s="27" t="n">
+      <c r="F42" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="G42" s="26" t="inlineStr"/>
-      <c r="H42" s="26" t="inlineStr"/>
-      <c r="I42" s="26" t="inlineStr"/>
-      <c r="J42" s="26" t="inlineStr"/>
-      <c r="K42" s="27" t="n">
+      <c r="G42" s="24" t="inlineStr"/>
+      <c r="H42" s="24" t="inlineStr"/>
+      <c r="I42" s="24" t="inlineStr"/>
+      <c r="J42" s="24" t="inlineStr"/>
+      <c r="K42" s="25" t="n">
         <v>623</v>
       </c>
-      <c r="L42" s="28" t="n">
+      <c r="L42" s="26" t="n">
         <v>0.65</v>
       </c>
-      <c r="M42" s="27" t="n">
+      <c r="M42" s="25" t="n">
         <v>402</v>
       </c>
-      <c r="N42" s="26" t="inlineStr"/>
-      <c r="O42" s="26" t="inlineStr"/>
-      <c r="P42" s="26" t="inlineStr"/>
-      <c r="Q42" s="26" t="inlineStr"/>
+      <c r="N42" s="24" t="inlineStr"/>
+      <c r="O42" s="24" t="inlineStr"/>
+      <c r="P42" s="24" t="inlineStr"/>
+      <c r="Q42" s="24" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="24" t="inlineStr"/>
-      <c r="B43" s="25" t="inlineStr">
+      <c r="A43" s="22" t="inlineStr"/>
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Dịch vụ toàn phần</t>
         </is>
       </c>
-      <c r="C43" s="26" t="inlineStr"/>
-      <c r="D43" s="27" t="n">
+      <c r="C43" s="24" t="inlineStr"/>
+      <c r="D43" s="25" t="n">
         <v>46</v>
       </c>
-      <c r="E43" s="28" t="n">
+      <c r="E43" s="26" t="n">
         <v>0.78</v>
       </c>
-      <c r="F43" s="27" t="n">
+      <c r="F43" s="25" t="n">
         <v>36</v>
       </c>
-      <c r="G43" s="26" t="inlineStr"/>
-      <c r="H43" s="26" t="inlineStr"/>
-      <c r="I43" s="26" t="inlineStr"/>
-      <c r="J43" s="26" t="inlineStr"/>
-      <c r="K43" s="27" t="n">
+      <c r="G43" s="24" t="inlineStr"/>
+      <c r="H43" s="24" t="inlineStr"/>
+      <c r="I43" s="24" t="inlineStr"/>
+      <c r="J43" s="24" t="inlineStr"/>
+      <c r="K43" s="25" t="n">
         <v>424</v>
       </c>
-      <c r="L43" s="28" t="n">
+      <c r="L43" s="26" t="n">
         <v>0.67</v>
       </c>
-      <c r="M43" s="27" t="n">
+      <c r="M43" s="25" t="n">
         <v>283</v>
       </c>
-      <c r="N43" s="26" t="inlineStr"/>
-      <c r="O43" s="26" t="inlineStr"/>
-      <c r="P43" s="26" t="inlineStr"/>
-      <c r="Q43" s="26" t="inlineStr"/>
+      <c r="N43" s="24" t="inlineStr"/>
+      <c r="O43" s="24" t="inlineStr"/>
+      <c r="P43" s="24" t="inlineStr"/>
+      <c r="Q43" s="24" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="24" t="inlineStr"/>
-      <c r="B44" s="25" t="inlineStr">
+      <c r="A44" s="22" t="inlineStr"/>
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">    Bán lẻ</t>
         </is>
       </c>
-      <c r="C44" s="26" t="inlineStr"/>
-      <c r="D44" s="27" t="n">
+      <c r="C44" s="24" t="inlineStr"/>
+      <c r="D44" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="E44" s="28" t="n">
+      <c r="E44" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="F44" s="27" t="n">
+      <c r="F44" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="G44" s="26" t="inlineStr"/>
-      <c r="H44" s="26" t="inlineStr"/>
-      <c r="I44" s="26" t="inlineStr"/>
-      <c r="J44" s="26" t="inlineStr"/>
-      <c r="K44" s="27" t="n">
+      <c r="G44" s="24" t="inlineStr"/>
+      <c r="H44" s="24" t="inlineStr"/>
+      <c r="I44" s="24" t="inlineStr"/>
+      <c r="J44" s="24" t="inlineStr"/>
+      <c r="K44" s="25" t="n">
         <v>304</v>
       </c>
-      <c r="L44" s="28" t="n">
+      <c r="L44" s="26" t="n">
         <v>0.17</v>
       </c>
-      <c r="M44" s="27" t="n">
+      <c r="M44" s="25" t="n">
         <v>52</v>
       </c>
-      <c r="N44" s="26" t="inlineStr"/>
-      <c r="O44" s="26" t="inlineStr"/>
-      <c r="P44" s="26" t="inlineStr"/>
-      <c r="Q44" s="26" t="inlineStr"/>
+      <c r="N44" s="24" t="inlineStr"/>
+      <c r="O44" s="24" t="inlineStr"/>
+      <c r="P44" s="24" t="inlineStr"/>
+      <c r="Q44" s="24" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="31" t="inlineStr">
@@ -2464,32 +2523,44 @@
         </is>
       </c>
       <c r="C45" s="33" t="n">
-        <v>83000</v>
-      </c>
-      <c r="D45" s="34" t="inlineStr"/>
-      <c r="E45" s="35" t="n">
+        <v>93000</v>
+      </c>
+      <c r="D45" s="33" t="n">
+        <v>43128</v>
+      </c>
+      <c r="E45" s="34" t="n">
         <v>0.15</v>
       </c>
-      <c r="F45" s="34" t="inlineStr"/>
+      <c r="F45" s="33" t="n">
+        <v>6309</v>
+      </c>
       <c r="G45" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="H45" s="34" t="inlineStr"/>
+      <c r="H45" s="33" t="n">
+        <v>7085</v>
+      </c>
       <c r="I45" s="33" t="n">
         <v>1161</v>
       </c>
       <c r="J45" s="33" t="n">
         <v>830</v>
       </c>
-      <c r="K45" s="34" t="inlineStr"/>
-      <c r="L45" s="35" t="n">
+      <c r="K45" s="33" t="n">
+        <v>208724</v>
+      </c>
+      <c r="L45" s="34" t="n">
         <v>0.23</v>
       </c>
-      <c r="M45" s="34" t="inlineStr"/>
+      <c r="M45" s="33" t="n">
+        <v>47249</v>
+      </c>
       <c r="N45" s="33" t="n">
         <v>335</v>
       </c>
-      <c r="O45" s="34" t="inlineStr"/>
+      <c r="O45" s="33" t="n">
+        <v>50756</v>
+      </c>
       <c r="P45" s="33" t="n">
         <v>8033</v>
       </c>
@@ -2527,79 +2598,79 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="36" t="inlineStr">
+      <c r="B2" s="35" t="inlineStr">
         <is>
           <t>HƯỚNG DẪN NHẬP LIỆU VÀ KẾT NỐI TỰ ĐỘNG VÀO DASHBOARD TẬP ĐOÀN VPS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="37" t="inlineStr">
+      <c r="B4" s="36" t="inlineStr">
         <is>
           <t>1. Nguyên tắc cấu trúc:</t>
         </is>
       </c>
-      <c r="C4" s="38" t="inlineStr">
+      <c r="C4" s="37" t="inlineStr">
         <is>
           <t>Mỗi dòng chỉ tiêu có mã STT và Tên nội dung tương ứng để hệ thống nhận diện.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="37" t="inlineStr">
+      <c r="B5" s="36" t="inlineStr">
         <is>
           <t>2. Nhập số liệu các tháng tiếp theo:</t>
         </is>
       </c>
-      <c r="C5" s="38" t="inlineStr">
+      <c r="C5" s="37" t="inlineStr">
         <is>
           <t>Bạn có thể nhập trực tiếp vào sheet này khi đến kỳ báo cáo mới (VD: Tháng 8, Tháng 9...) hoặc nhân bản (Duplicate) sheet này thành các tab: Thang_08, Thang_09...</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="36" t="inlineStr">
         <is>
           <t>3. Tải file lên Google Drive:</t>
         </is>
       </c>
-      <c r="C6" s="38" t="inlineStr">
+      <c r="C6" s="37" t="inlineStr">
         <is>
           <t>Sau khi điền số liệu, tải file này lên Google Drive cá nhân hoặc Google Drive của tập đoàn.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="37" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
         <is>
           <t>4. Mở bằng Google Sheets:</t>
         </is>
       </c>
-      <c r="C7" s="38" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>Nhấp chuột phải vào file trên Drive -&gt; Chọn 'Mở bằng Google Trang tính' (Open with Google Sheets).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="37" t="inlineStr">
+      <c r="B8" s="36" t="inlineStr">
         <is>
           <t>5. Chia sẻ quyền xem:</t>
         </is>
       </c>
-      <c r="C8" s="38" t="inlineStr">
+      <c r="C8" s="37" t="inlineStr">
         <is>
           <t>Nhấn nút 'Chia sẻ' ở góc phải trên -&gt; Chọn 'Bất kỳ ai có đường liên kết' -&gt; Quyền 'Người xem'.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>6. Kết nối vào Dashboard:</t>
         </is>
       </c>
-      <c r="C9" s="38" t="inlineStr">
+      <c r="C9" s="37" t="inlineStr">
         <is>
           <t>Sao chép đường link Google Sheets -&gt; Vào mục '13. Kết Quả KD' trên Dashboard -&gt; Nhấn 'Kết nối Google Sheet' -&gt; Dán link và nhấn Lưu. Hệ thống sẽ tự động quét số liệu ngay lập tức!</t>
         </is>

</xml_diff>